<commit_message>
category colours and shift-based positioning
Mapped drink categories to colours and organised sales observations by working shift
</commit_message>
<xml_diff>
--- a/Behind_the_Bar_Data.xlsx
+++ b/Behind_the_Bar_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Dear Data 100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2206A8-C704-46F1-A3BB-A39DF5028954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B225DDFD-3F53-47F7-8766-E0AD23FCF0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="65">
   <si>
     <t>Category</t>
   </si>
@@ -146,9 +146,6 @@
   </si>
   <si>
     <t>Cocktail</t>
-  </si>
-  <si>
-    <t>Mixed Drink</t>
   </si>
   <si>
     <t>Wine</t>
@@ -248,7 +245,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -279,6 +276,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -292,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -300,6 +303,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -736,7 +740,7 @@
         <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -747,7 +751,7 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -890,7 +894,7 @@
         <v>29</v>
       </c>
       <c r="B28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -901,7 +905,7 @@
         <v>30</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -912,7 +916,7 @@
         <v>31</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -923,7 +927,7 @@
         <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -931,7 +935,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
         <v>33</v>
@@ -942,7 +946,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B33" t="s">
         <v>33</v>
@@ -953,7 +957,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B34" t="s">
         <v>33</v>
@@ -964,10 +968,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B35" t="s">
         <v>52</v>
-      </c>
-      <c r="B35" t="s">
-        <v>53</v>
       </c>
       <c r="C35">
         <v>4</v>
@@ -975,7 +979,7 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B36" t="s">
         <v>36</v>
@@ -986,10 +990,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C37">
         <v>4</v>
@@ -997,10 +1001,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C38">
         <v>4</v>
@@ -1008,10 +1012,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C39">
         <v>3</v>
@@ -1019,10 +1023,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" t="s">
         <v>56</v>
-      </c>
-      <c r="B40" t="s">
-        <v>57</v>
       </c>
       <c r="C40">
         <v>3</v>
@@ -1030,10 +1034,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -1041,10 +1045,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -1052,10 +1056,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -1063,10 +1067,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -1074,10 +1078,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -1085,10 +1089,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -1096,10 +1100,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -1107,10 +1111,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -1118,10 +1122,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -1129,10 +1133,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B50" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1140,10 +1144,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B51" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -1188,11 +1192,11 @@
     <col min="32" max="32" width="11.33203125" customWidth="1"/>
     <col min="33" max="33" width="10.5546875" customWidth="1"/>
     <col min="34" max="34" width="12.77734375" customWidth="1"/>
-    <col min="37" max="37" width="13" customWidth="1"/>
-    <col min="38" max="38" width="18.109375" customWidth="1"/>
-    <col min="39" max="39" width="15.77734375" customWidth="1"/>
-    <col min="40" max="40" width="18" customWidth="1"/>
-    <col min="41" max="41" width="17.77734375" customWidth="1"/>
+    <col min="37" max="37" width="17.77734375" customWidth="1"/>
+    <col min="38" max="38" width="13" customWidth="1"/>
+    <col min="39" max="39" width="18.109375" customWidth="1"/>
+    <col min="40" max="40" width="15.77734375" customWidth="1"/>
+    <col min="41" max="41" width="18" customWidth="1"/>
     <col min="42" max="42" width="9" customWidth="1"/>
     <col min="45" max="45" width="11" customWidth="1"/>
     <col min="46" max="46" width="11.88671875" customWidth="1"/>
@@ -1291,85 +1295,85 @@
         <v>28</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AD1" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AE1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AF1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AG1" s="4" t="s">
+      <c r="AG1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AH1" s="4" t="s">
+      <c r="AH1" s="7" t="s">
         <v>32</v>
       </c>
       <c r="AI1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AJ1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK1" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="AK1" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="AL1" s="5" t="s">
         <v>60</v>
       </c>
       <c r="AM1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AN1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="AO1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AN1" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="AO1" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="AP1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="AQ1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AR1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AS1" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="AQ1" s="6" t="s">
+      <c r="AT1" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AU1" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AV1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="AW1" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="AX1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="AR1" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AS1" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="AT1" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="AU1" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="AV1" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW1" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="AX1" s="6" t="s">
+      <c r="AY1" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="AY1" s="6" t="s">
+      <c r="AZ1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="AZ1" s="6" t="s">
-        <v>47</v>
-      </c>
       <c r="BA1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BB1" t="s">
         <v>62</v>
       </c>
-      <c r="BB1" t="s">
+      <c r="BC1" t="s">
         <v>63</v>
-      </c>
-      <c r="BC1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.3">
@@ -1463,16 +1467,16 @@
       <c r="AD2" s="3">
         <v>0</v>
       </c>
-      <c r="AE2" s="4">
+      <c r="AE2" s="7">
         <v>24</v>
       </c>
-      <c r="AF2" s="4">
+      <c r="AF2" s="7">
         <v>6</v>
       </c>
-      <c r="AG2" s="4">
-        <v>1</v>
-      </c>
-      <c r="AH2" s="4">
+      <c r="AG2" s="7">
+        <v>1</v>
+      </c>
+      <c r="AH2" s="7">
         <v>2</v>
       </c>
       <c r="AI2" s="4">
@@ -1481,7 +1485,7 @@
       <c r="AJ2" s="4">
         <v>4</v>
       </c>
-      <c r="AK2" s="5">
+      <c r="AK2" s="4">
         <v>0</v>
       </c>
       <c r="AL2" s="5">
@@ -1493,7 +1497,7 @@
       <c r="AN2" s="5">
         <v>0</v>
       </c>
-      <c r="AO2" s="6">
+      <c r="AO2" s="5">
         <v>0</v>
       </c>
       <c r="AP2" s="6">
@@ -1633,16 +1637,16 @@
       <c r="AD3" s="3">
         <v>0</v>
       </c>
-      <c r="AE3" s="4">
+      <c r="AE3" s="7">
         <v>12</v>
       </c>
-      <c r="AF3" s="4">
-        <v>2</v>
-      </c>
-      <c r="AG3" s="4">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="4">
+      <c r="AF3" s="7">
+        <v>2</v>
+      </c>
+      <c r="AG3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="7">
         <v>0</v>
       </c>
       <c r="AI3" s="4">
@@ -1651,7 +1655,7 @@
       <c r="AJ3" s="4">
         <v>2</v>
       </c>
-      <c r="AK3" s="5">
+      <c r="AK3" s="4">
         <v>0</v>
       </c>
       <c r="AL3" s="5">
@@ -1663,7 +1667,7 @@
       <c r="AN3" s="5">
         <v>0</v>
       </c>
-      <c r="AO3" s="6">
+      <c r="AO3" s="5">
         <v>0</v>
       </c>
       <c r="AP3" s="6">
@@ -1803,16 +1807,16 @@
       <c r="AD4" s="3">
         <v>0</v>
       </c>
-      <c r="AE4" s="4">
+      <c r="AE4" s="7">
         <v>84</v>
       </c>
-      <c r="AF4" s="4">
+      <c r="AF4" s="7">
         <v>18</v>
       </c>
-      <c r="AG4" s="4">
+      <c r="AG4" s="7">
         <v>6</v>
       </c>
-      <c r="AH4" s="4">
+      <c r="AH4" s="7">
         <v>36</v>
       </c>
       <c r="AI4" s="4">
@@ -1821,7 +1825,7 @@
       <c r="AJ4" s="4">
         <v>48</v>
       </c>
-      <c r="AK4" s="5">
+      <c r="AK4" s="4">
         <v>0</v>
       </c>
       <c r="AL4" s="5">
@@ -1833,7 +1837,7 @@
       <c r="AN4" s="5">
         <v>0</v>
       </c>
-      <c r="AO4" s="6">
+      <c r="AO4" s="5">
         <v>0</v>
       </c>
       <c r="AP4" s="6">
@@ -1973,16 +1977,16 @@
       <c r="AD5" s="3">
         <v>0</v>
       </c>
-      <c r="AE5" s="4">
+      <c r="AE5" s="7">
         <v>50</v>
       </c>
-      <c r="AF5" s="4">
+      <c r="AF5" s="7">
         <v>10</v>
       </c>
-      <c r="AG5" s="4">
+      <c r="AG5" s="7">
         <v>4</v>
       </c>
-      <c r="AH5" s="4">
+      <c r="AH5" s="7">
         <v>6</v>
       </c>
       <c r="AI5" s="4">
@@ -1991,20 +1995,20 @@
       <c r="AJ5" s="4">
         <v>30</v>
       </c>
-      <c r="AK5" s="5">
+      <c r="AK5" s="4">
+        <v>1</v>
+      </c>
+      <c r="AL5" s="5">
         <v>4</v>
       </c>
-      <c r="AL5" s="5">
-        <v>0</v>
-      </c>
       <c r="AM5" s="5">
         <v>0</v>
       </c>
       <c r="AN5" s="5">
         <v>0</v>
       </c>
-      <c r="AO5" s="6">
-        <v>1</v>
+      <c r="AO5" s="5">
+        <v>0</v>
       </c>
       <c r="AP5" s="6">
         <v>15</v>
@@ -2143,16 +2147,16 @@
       <c r="AD6" s="3">
         <v>0</v>
       </c>
-      <c r="AE6" s="4">
+      <c r="AE6" s="7">
         <v>70</v>
       </c>
-      <c r="AF6" s="4">
+      <c r="AF6" s="7">
         <v>8</v>
       </c>
-      <c r="AG6" s="4">
-        <v>2</v>
-      </c>
-      <c r="AH6" s="4">
+      <c r="AG6" s="7">
+        <v>2</v>
+      </c>
+      <c r="AH6" s="7">
         <v>4</v>
       </c>
       <c r="AI6" s="4">
@@ -2161,19 +2165,19 @@
       <c r="AJ6" s="4">
         <v>20</v>
       </c>
-      <c r="AK6" s="5">
+      <c r="AK6" s="4">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="5">
         <v>6</v>
       </c>
-      <c r="AL6" s="5">
-        <v>0</v>
-      </c>
       <c r="AM6" s="5">
         <v>0</v>
       </c>
       <c r="AN6" s="5">
         <v>0</v>
       </c>
-      <c r="AO6" s="6">
+      <c r="AO6" s="5">
         <v>0</v>
       </c>
       <c r="AP6" s="6">
@@ -2313,16 +2317,16 @@
       <c r="AD7" s="3">
         <v>4</v>
       </c>
-      <c r="AE7" s="4">
+      <c r="AE7" s="7">
         <v>12</v>
       </c>
-      <c r="AF7" s="4">
+      <c r="AF7" s="7">
         <v>6</v>
       </c>
-      <c r="AG7" s="4">
-        <v>1</v>
-      </c>
-      <c r="AH7" s="4">
+      <c r="AG7" s="7">
+        <v>1</v>
+      </c>
+      <c r="AH7" s="7">
         <v>20</v>
       </c>
       <c r="AI7" s="4">
@@ -2331,8 +2335,8 @@
       <c r="AJ7" s="4">
         <v>6</v>
       </c>
-      <c r="AK7" s="5">
-        <v>0</v>
+      <c r="AK7" s="4">
+        <v>2</v>
       </c>
       <c r="AL7" s="5">
         <v>0</v>
@@ -2343,8 +2347,8 @@
       <c r="AN7" s="5">
         <v>0</v>
       </c>
-      <c r="AO7" s="6">
-        <v>2</v>
+      <c r="AO7" s="5">
+        <v>0</v>
       </c>
       <c r="AP7" s="6">
         <v>10</v>
@@ -2483,16 +2487,16 @@
       <c r="AD8" s="3">
         <v>0</v>
       </c>
-      <c r="AE8" s="4">
+      <c r="AE8" s="7">
         <v>36</v>
       </c>
-      <c r="AF8" s="4">
+      <c r="AF8" s="7">
         <v>24</v>
       </c>
-      <c r="AG8" s="4">
+      <c r="AG8" s="7">
         <v>4</v>
       </c>
-      <c r="AH8" s="4">
+      <c r="AH8" s="7">
         <v>4</v>
       </c>
       <c r="AI8" s="4">
@@ -2501,7 +2505,7 @@
       <c r="AJ8" s="4">
         <v>10</v>
       </c>
-      <c r="AK8" s="5">
+      <c r="AK8" s="4">
         <v>0</v>
       </c>
       <c r="AL8" s="5">
@@ -2513,7 +2517,7 @@
       <c r="AN8" s="5">
         <v>0</v>
       </c>
-      <c r="AO8" s="6">
+      <c r="AO8" s="5">
         <v>0</v>
       </c>
       <c r="AP8" s="6">
@@ -2653,16 +2657,16 @@
       <c r="AD9" s="3">
         <v>1</v>
       </c>
-      <c r="AE9" s="4">
+      <c r="AE9" s="7">
         <v>72</v>
       </c>
-      <c r="AF9" s="4">
+      <c r="AF9" s="7">
         <v>36</v>
       </c>
-      <c r="AG9" s="4">
+      <c r="AG9" s="7">
         <v>10</v>
       </c>
-      <c r="AH9" s="4">
+      <c r="AH9" s="7">
         <v>6</v>
       </c>
       <c r="AI9" s="4">
@@ -2671,20 +2675,20 @@
       <c r="AJ9" s="4">
         <v>12</v>
       </c>
-      <c r="AK9" s="5">
-        <v>0</v>
+      <c r="AK9" s="4">
+        <v>1</v>
       </c>
       <c r="AL9" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM9" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN9" s="5">
         <v>0</v>
       </c>
-      <c r="AO9" s="6">
-        <v>1</v>
+      <c r="AO9" s="5">
+        <v>0</v>
       </c>
       <c r="AP9" s="6">
         <v>20</v>
@@ -2823,16 +2827,16 @@
       <c r="AD10" s="3">
         <v>1</v>
       </c>
-      <c r="AE10" s="4">
+      <c r="AE10" s="7">
         <v>50</v>
       </c>
-      <c r="AF10" s="4">
+      <c r="AF10" s="7">
         <v>26</v>
       </c>
-      <c r="AG10" s="4">
-        <v>0</v>
-      </c>
-      <c r="AH10" s="4">
+      <c r="AG10" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="7">
         <v>16</v>
       </c>
       <c r="AI10" s="4">
@@ -2841,20 +2845,20 @@
       <c r="AJ10" s="4">
         <v>0</v>
       </c>
-      <c r="AK10" s="5">
-        <v>0</v>
+      <c r="AK10" s="4">
+        <v>2</v>
       </c>
       <c r="AL10" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM10" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN10" s="5">
         <v>0</v>
       </c>
-      <c r="AO10" s="6">
-        <v>2</v>
+      <c r="AO10" s="5">
+        <v>0</v>
       </c>
       <c r="AP10" s="6">
         <v>6</v>
@@ -2993,16 +2997,16 @@
       <c r="AD11" s="3">
         <v>2</v>
       </c>
-      <c r="AE11" s="4">
+      <c r="AE11" s="7">
         <v>42</v>
       </c>
-      <c r="AF11" s="4">
+      <c r="AF11" s="7">
         <v>24</v>
       </c>
-      <c r="AG11" s="4">
-        <v>0</v>
-      </c>
-      <c r="AH11" s="4">
+      <c r="AG11" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH11" s="7">
         <v>18</v>
       </c>
       <c r="AI11" s="4">
@@ -3011,8 +3015,8 @@
       <c r="AJ11" s="4">
         <v>20</v>
       </c>
-      <c r="AK11" s="5">
-        <v>0</v>
+      <c r="AK11" s="4">
+        <v>1</v>
       </c>
       <c r="AL11" s="5">
         <v>0</v>
@@ -3023,8 +3027,8 @@
       <c r="AN11" s="5">
         <v>0</v>
       </c>
-      <c r="AO11" s="6">
-        <v>1</v>
+      <c r="AO11" s="5">
+        <v>0</v>
       </c>
       <c r="AP11" s="6">
         <v>22</v>
@@ -3104,17 +3108,17 @@
       <c r="AB12" s="3"/>
       <c r="AC12" s="3"/>
       <c r="AD12" s="3"/>
-      <c r="AE12" s="4"/>
-      <c r="AF12" s="4"/>
-      <c r="AG12" s="4"/>
-      <c r="AH12" s="4"/>
+      <c r="AE12" s="7"/>
+      <c r="AF12" s="7"/>
+      <c r="AG12" s="7"/>
+      <c r="AH12" s="7"/>
       <c r="AI12" s="4"/>
       <c r="AJ12" s="4"/>
-      <c r="AK12" s="5"/>
+      <c r="AK12" s="4"/>
       <c r="AL12" s="5"/>
       <c r="AM12" s="5"/>
       <c r="AN12" s="5"/>
-      <c r="AO12" s="6"/>
+      <c r="AO12" s="5"/>
       <c r="AP12" s="6"/>
       <c r="AQ12" s="6"/>
       <c r="AR12" s="6"/>
@@ -3171,17 +3175,17 @@
       <c r="AB13" s="3"/>
       <c r="AC13" s="3"/>
       <c r="AD13" s="3"/>
-      <c r="AE13" s="4"/>
-      <c r="AF13" s="4"/>
-      <c r="AG13" s="4"/>
-      <c r="AH13" s="4"/>
+      <c r="AE13" s="7"/>
+      <c r="AF13" s="7"/>
+      <c r="AG13" s="7"/>
+      <c r="AH13" s="7"/>
       <c r="AI13" s="4"/>
       <c r="AJ13" s="4"/>
-      <c r="AK13" s="5"/>
+      <c r="AK13" s="4"/>
       <c r="AL13" s="5"/>
       <c r="AM13" s="5"/>
       <c r="AN13" s="5"/>
-      <c r="AO13" s="6"/>
+      <c r="AO13" s="5"/>
       <c r="AP13" s="6"/>
       <c r="AQ13" s="6"/>
       <c r="AR13" s="6"/>
@@ -3238,17 +3242,17 @@
       <c r="AB14" s="3"/>
       <c r="AC14" s="3"/>
       <c r="AD14" s="3"/>
-      <c r="AE14" s="4"/>
-      <c r="AF14" s="4"/>
-      <c r="AG14" s="4"/>
-      <c r="AH14" s="4"/>
+      <c r="AE14" s="7"/>
+      <c r="AF14" s="7"/>
+      <c r="AG14" s="7"/>
+      <c r="AH14" s="7"/>
       <c r="AI14" s="4"/>
       <c r="AJ14" s="4"/>
-      <c r="AK14" s="5"/>
+      <c r="AK14" s="4"/>
       <c r="AL14" s="5"/>
       <c r="AM14" s="5"/>
       <c r="AN14" s="5"/>
-      <c r="AO14" s="6"/>
+      <c r="AO14" s="5"/>
       <c r="AP14" s="6"/>
       <c r="AQ14" s="6"/>
       <c r="AR14" s="6"/>
@@ -3305,17 +3309,17 @@
       <c r="AB15" s="3"/>
       <c r="AC15" s="3"/>
       <c r="AD15" s="3"/>
-      <c r="AE15" s="4"/>
-      <c r="AF15" s="4"/>
-      <c r="AG15" s="4"/>
-      <c r="AH15" s="4"/>
+      <c r="AE15" s="7"/>
+      <c r="AF15" s="7"/>
+      <c r="AG15" s="7"/>
+      <c r="AH15" s="7"/>
       <c r="AI15" s="4"/>
       <c r="AJ15" s="4"/>
-      <c r="AK15" s="5"/>
+      <c r="AK15" s="4"/>
       <c r="AL15" s="5"/>
       <c r="AM15" s="5"/>
       <c r="AN15" s="5"/>
-      <c r="AO15" s="6"/>
+      <c r="AO15" s="5"/>
       <c r="AP15" s="6"/>
       <c r="AQ15" s="6"/>
       <c r="AR15" s="6"/>
@@ -3372,17 +3376,17 @@
       <c r="AB16" s="3"/>
       <c r="AC16" s="3"/>
       <c r="AD16" s="3"/>
-      <c r="AE16" s="4"/>
-      <c r="AF16" s="4"/>
-      <c r="AG16" s="4"/>
-      <c r="AH16" s="4"/>
+      <c r="AE16" s="7"/>
+      <c r="AF16" s="7"/>
+      <c r="AG16" s="7"/>
+      <c r="AH16" s="7"/>
       <c r="AI16" s="4"/>
       <c r="AJ16" s="4"/>
-      <c r="AK16" s="5"/>
+      <c r="AK16" s="4"/>
       <c r="AL16" s="5"/>
       <c r="AM16" s="5"/>
       <c r="AN16" s="5"/>
-      <c r="AO16" s="6"/>
+      <c r="AO16" s="5"/>
       <c r="AP16" s="6"/>
       <c r="AQ16" s="6"/>
       <c r="AR16" s="6"/>
@@ -3436,17 +3440,17 @@
       <c r="AB17" s="3"/>
       <c r="AC17" s="3"/>
       <c r="AD17" s="3"/>
-      <c r="AE17" s="4"/>
-      <c r="AF17" s="4"/>
-      <c r="AG17" s="4"/>
-      <c r="AH17" s="4"/>
+      <c r="AE17" s="7"/>
+      <c r="AF17" s="7"/>
+      <c r="AG17" s="7"/>
+      <c r="AH17" s="7"/>
       <c r="AI17" s="4"/>
       <c r="AJ17" s="4"/>
-      <c r="AK17" s="5"/>
+      <c r="AK17" s="4"/>
       <c r="AL17" s="5"/>
       <c r="AM17" s="5"/>
       <c r="AN17" s="5"/>
-      <c r="AO17" s="6"/>
+      <c r="AO17" s="5"/>
       <c r="AP17" s="6"/>
       <c r="AQ17" s="6"/>
       <c r="AR17" s="6"/>
@@ -3459,13 +3463,13 @@
       <c r="AY17" s="6"/>
       <c r="AZ17" s="6"/>
       <c r="BA17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="BB17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="BC17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="3:55" x14ac:dyDescent="0.3">
@@ -3497,17 +3501,17 @@
       <c r="AB18" s="3"/>
       <c r="AC18" s="3"/>
       <c r="AD18" s="3"/>
-      <c r="AE18" s="4"/>
-      <c r="AF18" s="4"/>
-      <c r="AG18" s="4"/>
-      <c r="AH18" s="4"/>
+      <c r="AE18" s="7"/>
+      <c r="AF18" s="7"/>
+      <c r="AG18" s="7"/>
+      <c r="AH18" s="7"/>
       <c r="AI18" s="4"/>
       <c r="AJ18" s="4"/>
-      <c r="AK18" s="5"/>
+      <c r="AK18" s="4"/>
       <c r="AL18" s="5"/>
       <c r="AM18" s="5"/>
       <c r="AN18" s="5"/>
-      <c r="AO18" s="6"/>
+      <c r="AO18" s="5"/>
       <c r="AP18" s="6"/>
       <c r="AQ18" s="6"/>
       <c r="AR18" s="6"/>
@@ -3561,17 +3565,17 @@
       <c r="AB19" s="3"/>
       <c r="AC19" s="3"/>
       <c r="AD19" s="3"/>
-      <c r="AE19" s="4"/>
-      <c r="AF19" s="4"/>
-      <c r="AG19" s="4"/>
-      <c r="AH19" s="4"/>
+      <c r="AE19" s="7"/>
+      <c r="AF19" s="7"/>
+      <c r="AG19" s="7"/>
+      <c r="AH19" s="7"/>
       <c r="AI19" s="4"/>
       <c r="AJ19" s="4"/>
-      <c r="AK19" s="5"/>
+      <c r="AK19" s="4"/>
       <c r="AL19" s="5"/>
       <c r="AM19" s="5"/>
       <c r="AN19" s="5"/>
-      <c r="AO19" s="6"/>
+      <c r="AO19" s="5"/>
       <c r="AP19" s="6"/>
       <c r="AQ19" s="6"/>
       <c r="AR19" s="6"/>
@@ -3613,17 +3617,17 @@
       <c r="AB20" s="3"/>
       <c r="AC20" s="3"/>
       <c r="AD20" s="3"/>
-      <c r="AE20" s="4"/>
-      <c r="AF20" s="4"/>
-      <c r="AG20" s="4"/>
-      <c r="AH20" s="4"/>
+      <c r="AE20" s="7"/>
+      <c r="AF20" s="7"/>
+      <c r="AG20" s="7"/>
+      <c r="AH20" s="7"/>
       <c r="AI20" s="4"/>
       <c r="AJ20" s="4"/>
-      <c r="AK20" s="5"/>
+      <c r="AK20" s="4"/>
       <c r="AL20" s="5"/>
       <c r="AM20" s="5"/>
       <c r="AN20" s="5"/>
-      <c r="AO20" s="6"/>
+      <c r="AO20" s="5"/>
       <c r="AP20" s="6"/>
       <c r="AQ20" s="6"/>
       <c r="AR20" s="6"/>

</xml_diff>

<commit_message>
24&25 Oct data entry
</commit_message>
<xml_diff>
--- a/Behind_the_Bar_Data.xlsx
+++ b/Behind_the_Bar_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Dear Data 100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B225DDFD-3F53-47F7-8766-E0AD23FCF0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C132B94-E230-49C4-BF6C-6CFC0DB86750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -295,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -304,6 +304,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2214,7 +2215,7 @@
         <v>0</v>
       </c>
       <c r="BA6">
-        <f t="shared" ref="BA6:BA16" si="0">SUM(C6:AZ6)</f>
+        <f>SUM(C6:AZ6)</f>
         <v>232</v>
       </c>
       <c r="BB6">
@@ -2384,7 +2385,7 @@
         <v>2</v>
       </c>
       <c r="BA7">
-        <f t="shared" si="0"/>
+        <f>SUM(C7:AZ7)</f>
         <v>110</v>
       </c>
       <c r="BB7">
@@ -2554,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="BA8">
-        <f t="shared" si="0"/>
+        <f>SUM(C8:AZ8)</f>
         <v>114</v>
       </c>
       <c r="BB8">
@@ -2724,7 +2725,7 @@
         <v>0</v>
       </c>
       <c r="BA9">
-        <f t="shared" si="0"/>
+        <f>SUM(C9:AZ9)</f>
         <v>209</v>
       </c>
       <c r="BB9">
@@ -2894,7 +2895,7 @@
         <v>1</v>
       </c>
       <c r="BA10">
-        <f t="shared" si="0"/>
+        <f>SUM(C10:AZ10)</f>
         <v>115</v>
       </c>
       <c r="BB10">
@@ -3064,7 +3065,7 @@
         <v>2</v>
       </c>
       <c r="BA11">
-        <f t="shared" si="0"/>
+        <f>SUM(C11:AZ11)</f>
         <v>201</v>
       </c>
       <c r="BB11">
@@ -3080,192 +3081,396 @@
       <c r="A12" s="1">
         <v>46319</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="3"/>
-      <c r="Y12" s="3"/>
-      <c r="Z12" s="3"/>
-      <c r="AA12" s="3"/>
-      <c r="AB12" s="3"/>
-      <c r="AC12" s="3"/>
-      <c r="AD12" s="3"/>
-      <c r="AE12" s="7"/>
-      <c r="AF12" s="7"/>
-      <c r="AG12" s="7"/>
-      <c r="AH12" s="7"/>
-      <c r="AI12" s="4"/>
-      <c r="AJ12" s="4"/>
-      <c r="AK12" s="4"/>
-      <c r="AL12" s="5"/>
-      <c r="AM12" s="5"/>
-      <c r="AN12" s="5"/>
-      <c r="AO12" s="5"/>
-      <c r="AP12" s="6"/>
-      <c r="AQ12" s="6"/>
-      <c r="AR12" s="6"/>
-      <c r="AS12" s="6"/>
-      <c r="AT12" s="6"/>
-      <c r="AU12" s="6"/>
-      <c r="AV12" s="6"/>
-      <c r="AW12" s="6"/>
-      <c r="AX12" s="6"/>
-      <c r="AY12" s="6"/>
-      <c r="AZ12" s="6"/>
+      <c r="B12">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3">
+        <v>3</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
+        <v>4</v>
+      </c>
+      <c r="F12" s="3">
+        <v>2</v>
+      </c>
+      <c r="G12" s="3">
+        <v>3</v>
+      </c>
+      <c r="H12" s="3">
+        <v>2</v>
+      </c>
+      <c r="I12" s="3">
+        <v>8</v>
+      </c>
+      <c r="J12" s="3">
+        <v>1</v>
+      </c>
+      <c r="K12" s="3">
+        <v>2</v>
+      </c>
+      <c r="L12" s="3">
+        <v>1</v>
+      </c>
+      <c r="M12" s="3">
+        <v>1</v>
+      </c>
+      <c r="N12" s="3">
+        <v>0</v>
+      </c>
+      <c r="O12" s="3">
+        <v>5</v>
+      </c>
+      <c r="P12" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3">
+        <v>2</v>
+      </c>
+      <c r="R12" s="3">
+        <v>1</v>
+      </c>
+      <c r="S12" s="3">
+        <v>0</v>
+      </c>
+      <c r="T12" s="3">
+        <v>2</v>
+      </c>
+      <c r="U12" s="3">
+        <v>2</v>
+      </c>
+      <c r="V12" s="3">
+        <v>1</v>
+      </c>
+      <c r="W12" s="3">
+        <v>1</v>
+      </c>
+      <c r="X12" s="3">
+        <v>2</v>
+      </c>
+      <c r="Y12" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="3">
+        <v>5</v>
+      </c>
+      <c r="AC12" s="3">
+        <v>2</v>
+      </c>
+      <c r="AD12" s="3">
+        <v>1</v>
+      </c>
+      <c r="AE12" s="7">
+        <v>90</v>
+      </c>
+      <c r="AF12" s="7">
+        <v>30</v>
+      </c>
+      <c r="AG12" s="7">
+        <v>6</v>
+      </c>
+      <c r="AH12" s="7">
+        <v>18</v>
+      </c>
+      <c r="AI12" s="4">
+        <v>4</v>
+      </c>
+      <c r="AJ12" s="4">
+        <v>12</v>
+      </c>
+      <c r="AK12" s="4">
+        <v>3</v>
+      </c>
+      <c r="AL12" s="5">
+        <v>1</v>
+      </c>
+      <c r="AM12" s="5">
+        <v>1</v>
+      </c>
+      <c r="AN12" s="5">
+        <v>1</v>
+      </c>
+      <c r="AO12" s="5">
+        <v>2</v>
+      </c>
+      <c r="AP12" s="6">
+        <v>24</v>
+      </c>
+      <c r="AQ12" s="6">
+        <v>10</v>
+      </c>
+      <c r="AR12" s="6">
+        <v>3</v>
+      </c>
+      <c r="AS12" s="6">
+        <v>1</v>
+      </c>
+      <c r="AT12" s="6">
+        <v>2</v>
+      </c>
+      <c r="AU12" s="6">
+        <v>4</v>
+      </c>
+      <c r="AV12" s="6">
+        <v>6</v>
+      </c>
+      <c r="AW12" s="6">
+        <v>1</v>
+      </c>
+      <c r="AX12" s="6">
+        <v>7</v>
+      </c>
+      <c r="AY12" s="6">
+        <v>5</v>
+      </c>
+      <c r="AZ12" s="6">
+        <v>4</v>
+      </c>
       <c r="BA12">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(C12:AZ12)</f>
+        <v>287</v>
       </c>
       <c r="BB12">
         <f>COUNTIF(C12:AZ12,0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BC12">
         <f>COUNTIF(C12:AZ12,"&gt;0")</f>
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:55" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>46320</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
-      <c r="X13" s="3"/>
-      <c r="Y13" s="3"/>
-      <c r="Z13" s="3"/>
-      <c r="AA13" s="3"/>
-      <c r="AB13" s="3"/>
-      <c r="AC13" s="3"/>
-      <c r="AD13" s="3"/>
-      <c r="AE13" s="7"/>
-      <c r="AF13" s="7"/>
-      <c r="AG13" s="7"/>
-      <c r="AH13" s="7"/>
-      <c r="AI13" s="4"/>
-      <c r="AJ13" s="4"/>
-      <c r="AK13" s="4"/>
-      <c r="AL13" s="5"/>
-      <c r="AM13" s="5"/>
-      <c r="AN13" s="5"/>
-      <c r="AO13" s="5"/>
-      <c r="AP13" s="6"/>
-      <c r="AQ13" s="6"/>
-      <c r="AR13" s="6"/>
-      <c r="AS13" s="6"/>
-      <c r="AT13" s="6"/>
-      <c r="AU13" s="6"/>
-      <c r="AV13" s="6"/>
-      <c r="AW13" s="6"/>
-      <c r="AX13" s="6"/>
-      <c r="AY13" s="6"/>
-      <c r="AZ13" s="6"/>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>2</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>1</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0</v>
+      </c>
+      <c r="L13" s="3">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3">
+        <v>0</v>
+      </c>
+      <c r="N13" s="3">
+        <v>0</v>
+      </c>
+      <c r="O13" s="3">
+        <v>4</v>
+      </c>
+      <c r="P13" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="3">
+        <v>0</v>
+      </c>
+      <c r="R13" s="3">
+        <v>0</v>
+      </c>
+      <c r="S13" s="3">
+        <v>0</v>
+      </c>
+      <c r="T13" s="3">
+        <v>0</v>
+      </c>
+      <c r="U13" s="3">
+        <v>0</v>
+      </c>
+      <c r="V13" s="3">
+        <v>0</v>
+      </c>
+      <c r="W13" s="3">
+        <v>0</v>
+      </c>
+      <c r="X13" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="3">
+        <v>6</v>
+      </c>
+      <c r="AE13" s="7">
+        <v>24</v>
+      </c>
+      <c r="AF13" s="7">
+        <v>6</v>
+      </c>
+      <c r="AG13" s="7">
+        <v>4</v>
+      </c>
+      <c r="AH13" s="7">
+        <v>24</v>
+      </c>
+      <c r="AI13" s="4">
+        <v>6</v>
+      </c>
+      <c r="AJ13" s="4">
+        <v>8</v>
+      </c>
+      <c r="AK13" s="4">
+        <v>1</v>
+      </c>
+      <c r="AL13" s="5">
+        <v>0</v>
+      </c>
+      <c r="AM13" s="5">
+        <v>2</v>
+      </c>
+      <c r="AN13" s="5">
+        <v>0</v>
+      </c>
+      <c r="AO13" s="5">
+        <v>0</v>
+      </c>
+      <c r="AP13" s="6">
+        <v>10</v>
+      </c>
+      <c r="AQ13" s="6">
+        <v>2</v>
+      </c>
+      <c r="AR13" s="6">
+        <v>1</v>
+      </c>
+      <c r="AS13" s="6">
+        <v>1</v>
+      </c>
+      <c r="AT13" s="6">
+        <v>2</v>
+      </c>
+      <c r="AU13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AV13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AW13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AX13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AY13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AZ13" s="6">
+        <v>0</v>
+      </c>
       <c r="BA13">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>SUM(C13:AZ13)</f>
+        <v>104</v>
       </c>
       <c r="BB13">
         <f>COUNTIF(C13:AZ13,0)</f>
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="BC13">
         <f>COUNTIF(C13:AZ13,"&gt;0")</f>
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
-        <v>46325</v>
-      </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-      <c r="X14" s="3"/>
-      <c r="Y14" s="3"/>
-      <c r="Z14" s="3"/>
-      <c r="AA14" s="3"/>
-      <c r="AB14" s="3"/>
-      <c r="AC14" s="3"/>
-      <c r="AD14" s="3"/>
-      <c r="AE14" s="7"/>
-      <c r="AF14" s="7"/>
-      <c r="AG14" s="7"/>
-      <c r="AH14" s="7"/>
-      <c r="AI14" s="4"/>
-      <c r="AJ14" s="4"/>
-      <c r="AK14" s="4"/>
-      <c r="AL14" s="5"/>
-      <c r="AM14" s="5"/>
-      <c r="AN14" s="5"/>
-      <c r="AO14" s="5"/>
-      <c r="AP14" s="6"/>
-      <c r="AQ14" s="6"/>
-      <c r="AR14" s="6"/>
-      <c r="AS14" s="6"/>
-      <c r="AT14" s="6"/>
-      <c r="AU14" s="6"/>
-      <c r="AV14" s="6"/>
-      <c r="AW14" s="6"/>
-      <c r="AX14" s="6"/>
-      <c r="AY14" s="6"/>
-      <c r="AZ14" s="6"/>
+      <c r="A14" s="1"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
+      <c r="X14" s="8"/>
+      <c r="Y14" s="8"/>
+      <c r="Z14" s="8"/>
+      <c r="AA14" s="8"/>
+      <c r="AB14" s="8"/>
+      <c r="AC14" s="8"/>
+      <c r="AD14" s="8"/>
+      <c r="AE14" s="8"/>
+      <c r="AF14" s="8"/>
+      <c r="AG14" s="8"/>
+      <c r="AH14" s="8"/>
+      <c r="AI14" s="8"/>
+      <c r="AJ14" s="8"/>
+      <c r="AK14" s="8"/>
+      <c r="AL14" s="8"/>
+      <c r="AM14" s="8"/>
+      <c r="AN14" s="8"/>
+      <c r="AO14" s="8"/>
+      <c r="AP14" s="8"/>
+      <c r="AQ14" s="8"/>
+      <c r="AR14" s="8"/>
+      <c r="AS14" s="8"/>
+      <c r="AT14" s="8"/>
+      <c r="AU14" s="8"/>
+      <c r="AV14" s="8"/>
+      <c r="AW14" s="8"/>
+      <c r="AX14" s="8"/>
+      <c r="AY14" s="8"/>
+      <c r="AZ14" s="8"/>
       <c r="BA14">
-        <f t="shared" si="0"/>
+        <f>SUM(C14:AZ14)</f>
         <v>0</v>
       </c>
       <c r="BB14">
@@ -3278,61 +3483,59 @@
       </c>
     </row>
     <row r="15" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
-        <v>46326</v>
-      </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
-      <c r="Y15" s="3"/>
-      <c r="Z15" s="3"/>
-      <c r="AA15" s="3"/>
-      <c r="AB15" s="3"/>
-      <c r="AC15" s="3"/>
-      <c r="AD15" s="3"/>
-      <c r="AE15" s="7"/>
-      <c r="AF15" s="7"/>
-      <c r="AG15" s="7"/>
-      <c r="AH15" s="7"/>
-      <c r="AI15" s="4"/>
-      <c r="AJ15" s="4"/>
-      <c r="AK15" s="4"/>
-      <c r="AL15" s="5"/>
-      <c r="AM15" s="5"/>
-      <c r="AN15" s="5"/>
-      <c r="AO15" s="5"/>
-      <c r="AP15" s="6"/>
-      <c r="AQ15" s="6"/>
-      <c r="AR15" s="6"/>
-      <c r="AS15" s="6"/>
-      <c r="AT15" s="6"/>
-      <c r="AU15" s="6"/>
-      <c r="AV15" s="6"/>
-      <c r="AW15" s="6"/>
-      <c r="AX15" s="6"/>
-      <c r="AY15" s="6"/>
-      <c r="AZ15" s="6"/>
+      <c r="A15" s="1"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="8"/>
+      <c r="V15" s="8"/>
+      <c r="W15" s="8"/>
+      <c r="X15" s="8"/>
+      <c r="Y15" s="8"/>
+      <c r="Z15" s="8"/>
+      <c r="AA15" s="8"/>
+      <c r="AB15" s="8"/>
+      <c r="AC15" s="8"/>
+      <c r="AD15" s="8"/>
+      <c r="AE15" s="8"/>
+      <c r="AF15" s="8"/>
+      <c r="AG15" s="8"/>
+      <c r="AH15" s="8"/>
+      <c r="AI15" s="8"/>
+      <c r="AJ15" s="8"/>
+      <c r="AK15" s="8"/>
+      <c r="AL15" s="8"/>
+      <c r="AM15" s="8"/>
+      <c r="AN15" s="8"/>
+      <c r="AO15" s="8"/>
+      <c r="AP15" s="8"/>
+      <c r="AQ15" s="8"/>
+      <c r="AR15" s="8"/>
+      <c r="AS15" s="8"/>
+      <c r="AT15" s="8"/>
+      <c r="AU15" s="8"/>
+      <c r="AV15" s="8"/>
+      <c r="AW15" s="8"/>
+      <c r="AX15" s="8"/>
+      <c r="AY15" s="8"/>
+      <c r="AZ15" s="8"/>
       <c r="BA15">
-        <f t="shared" si="0"/>
+        <f>SUM(C15:AZ15)</f>
         <v>0</v>
       </c>
       <c r="BB15">
@@ -3345,61 +3548,59 @@
       </c>
     </row>
     <row r="16" spans="1:55" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
-        <v>46327</v>
-      </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
-      <c r="S16" s="3"/>
-      <c r="T16" s="3"/>
-      <c r="U16" s="3"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
-      <c r="X16" s="3"/>
-      <c r="Y16" s="3"/>
-      <c r="Z16" s="3"/>
-      <c r="AA16" s="3"/>
-      <c r="AB16" s="3"/>
-      <c r="AC16" s="3"/>
-      <c r="AD16" s="3"/>
-      <c r="AE16" s="7"/>
-      <c r="AF16" s="7"/>
-      <c r="AG16" s="7"/>
-      <c r="AH16" s="7"/>
-      <c r="AI16" s="4"/>
-      <c r="AJ16" s="4"/>
-      <c r="AK16" s="4"/>
-      <c r="AL16" s="5"/>
-      <c r="AM16" s="5"/>
-      <c r="AN16" s="5"/>
-      <c r="AO16" s="5"/>
-      <c r="AP16" s="6"/>
-      <c r="AQ16" s="6"/>
-      <c r="AR16" s="6"/>
-      <c r="AS16" s="6"/>
-      <c r="AT16" s="6"/>
-      <c r="AU16" s="6"/>
-      <c r="AV16" s="6"/>
-      <c r="AW16" s="6"/>
-      <c r="AX16" s="6"/>
-      <c r="AY16" s="6"/>
-      <c r="AZ16" s="6"/>
+      <c r="A16" s="1"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="8"/>
+      <c r="V16" s="8"/>
+      <c r="W16" s="8"/>
+      <c r="X16" s="8"/>
+      <c r="Y16" s="8"/>
+      <c r="Z16" s="8"/>
+      <c r="AA16" s="8"/>
+      <c r="AB16" s="8"/>
+      <c r="AC16" s="8"/>
+      <c r="AD16" s="8"/>
+      <c r="AE16" s="8"/>
+      <c r="AF16" s="8"/>
+      <c r="AG16" s="8"/>
+      <c r="AH16" s="8"/>
+      <c r="AI16" s="8"/>
+      <c r="AJ16" s="8"/>
+      <c r="AK16" s="8"/>
+      <c r="AL16" s="8"/>
+      <c r="AM16" s="8"/>
+      <c r="AN16" s="8"/>
+      <c r="AO16" s="8"/>
+      <c r="AP16" s="8"/>
+      <c r="AQ16" s="8"/>
+      <c r="AR16" s="8"/>
+      <c r="AS16" s="8"/>
+      <c r="AT16" s="8"/>
+      <c r="AU16" s="8"/>
+      <c r="AV16" s="8"/>
+      <c r="AW16" s="8"/>
+      <c r="AX16" s="8"/>
+      <c r="AY16" s="8"/>
+      <c r="AZ16" s="8"/>
       <c r="BA16">
-        <f t="shared" si="0"/>
+        <f>SUM(C16:AZ16)</f>
         <v>0</v>
       </c>
       <c r="BB16">
@@ -3412,56 +3613,56 @@
       </c>
     </row>
     <row r="17" spans="3:55" x14ac:dyDescent="0.3">
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
-      <c r="X17" s="3"/>
-      <c r="Y17" s="3"/>
-      <c r="Z17" s="3"/>
-      <c r="AA17" s="3"/>
-      <c r="AB17" s="3"/>
-      <c r="AC17" s="3"/>
-      <c r="AD17" s="3"/>
-      <c r="AE17" s="7"/>
-      <c r="AF17" s="7"/>
-      <c r="AG17" s="7"/>
-      <c r="AH17" s="7"/>
-      <c r="AI17" s="4"/>
-      <c r="AJ17" s="4"/>
-      <c r="AK17" s="4"/>
-      <c r="AL17" s="5"/>
-      <c r="AM17" s="5"/>
-      <c r="AN17" s="5"/>
-      <c r="AO17" s="5"/>
-      <c r="AP17" s="6"/>
-      <c r="AQ17" s="6"/>
-      <c r="AR17" s="6"/>
-      <c r="AS17" s="6"/>
-      <c r="AT17" s="6"/>
-      <c r="AU17" s="6"/>
-      <c r="AV17" s="6"/>
-      <c r="AW17" s="6"/>
-      <c r="AX17" s="6"/>
-      <c r="AY17" s="6"/>
-      <c r="AZ17" s="6"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="8"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="8"/>
+      <c r="V17" s="8"/>
+      <c r="W17" s="8"/>
+      <c r="X17" s="8"/>
+      <c r="Y17" s="8"/>
+      <c r="Z17" s="8"/>
+      <c r="AA17" s="8"/>
+      <c r="AB17" s="8"/>
+      <c r="AC17" s="8"/>
+      <c r="AD17" s="8"/>
+      <c r="AE17" s="8"/>
+      <c r="AF17" s="8"/>
+      <c r="AG17" s="8"/>
+      <c r="AH17" s="8"/>
+      <c r="AI17" s="8"/>
+      <c r="AJ17" s="8"/>
+      <c r="AK17" s="8"/>
+      <c r="AL17" s="8"/>
+      <c r="AM17" s="8"/>
+      <c r="AN17" s="8"/>
+      <c r="AO17" s="8"/>
+      <c r="AP17" s="8"/>
+      <c r="AQ17" s="8"/>
+      <c r="AR17" s="8"/>
+      <c r="AS17" s="8"/>
+      <c r="AT17" s="8"/>
+      <c r="AU17" s="8"/>
+      <c r="AV17" s="8"/>
+      <c r="AW17" s="8"/>
+      <c r="AX17" s="8"/>
+      <c r="AY17" s="8"/>
+      <c r="AZ17" s="8"/>
       <c r="BA17" t="s">
         <v>64</v>
       </c>
@@ -3473,172 +3674,172 @@
       </c>
     </row>
     <row r="18" spans="3:55" x14ac:dyDescent="0.3">
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
-      <c r="Y18" s="3"/>
-      <c r="Z18" s="3"/>
-      <c r="AA18" s="3"/>
-      <c r="AB18" s="3"/>
-      <c r="AC18" s="3"/>
-      <c r="AD18" s="3"/>
-      <c r="AE18" s="7"/>
-      <c r="AF18" s="7"/>
-      <c r="AG18" s="7"/>
-      <c r="AH18" s="7"/>
-      <c r="AI18" s="4"/>
-      <c r="AJ18" s="4"/>
-      <c r="AK18" s="4"/>
-      <c r="AL18" s="5"/>
-      <c r="AM18" s="5"/>
-      <c r="AN18" s="5"/>
-      <c r="AO18" s="5"/>
-      <c r="AP18" s="6"/>
-      <c r="AQ18" s="6"/>
-      <c r="AR18" s="6"/>
-      <c r="AS18" s="6"/>
-      <c r="AT18" s="6"/>
-      <c r="AU18" s="6"/>
-      <c r="AV18" s="6"/>
-      <c r="AW18" s="6"/>
-      <c r="AX18" s="6"/>
-      <c r="AY18" s="6"/>
-      <c r="AZ18" s="6"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+      <c r="V18" s="8"/>
+      <c r="W18" s="8"/>
+      <c r="X18" s="8"/>
+      <c r="Y18" s="8"/>
+      <c r="Z18" s="8"/>
+      <c r="AA18" s="8"/>
+      <c r="AB18" s="8"/>
+      <c r="AC18" s="8"/>
+      <c r="AD18" s="8"/>
+      <c r="AE18" s="8"/>
+      <c r="AF18" s="8"/>
+      <c r="AG18" s="8"/>
+      <c r="AH18" s="8"/>
+      <c r="AI18" s="8"/>
+      <c r="AJ18" s="8"/>
+      <c r="AK18" s="8"/>
+      <c r="AL18" s="8"/>
+      <c r="AM18" s="8"/>
+      <c r="AN18" s="8"/>
+      <c r="AO18" s="8"/>
+      <c r="AP18" s="8"/>
+      <c r="AQ18" s="8"/>
+      <c r="AR18" s="8"/>
+      <c r="AS18" s="8"/>
+      <c r="AT18" s="8"/>
+      <c r="AU18" s="8"/>
+      <c r="AV18" s="8"/>
+      <c r="AW18" s="8"/>
+      <c r="AX18" s="8"/>
+      <c r="AY18" s="8"/>
+      <c r="AZ18" s="8"/>
       <c r="BA18">
         <f>SUM(C2:AZ16)</f>
-        <v>1604</v>
+        <v>1995</v>
       </c>
       <c r="BB18">
         <f>COUNTIF(C2:AZ16,0)</f>
-        <v>281</v>
+        <v>320</v>
       </c>
       <c r="BC18">
         <f>COUNTIF(C2:AZ16,"&gt;0")</f>
-        <v>219</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19" spans="3:55" x14ac:dyDescent="0.3">
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="3"/>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
-      <c r="Y19" s="3"/>
-      <c r="Z19" s="3"/>
-      <c r="AA19" s="3"/>
-      <c r="AB19" s="3"/>
-      <c r="AC19" s="3"/>
-      <c r="AD19" s="3"/>
-      <c r="AE19" s="7"/>
-      <c r="AF19" s="7"/>
-      <c r="AG19" s="7"/>
-      <c r="AH19" s="7"/>
-      <c r="AI19" s="4"/>
-      <c r="AJ19" s="4"/>
-      <c r="AK19" s="4"/>
-      <c r="AL19" s="5"/>
-      <c r="AM19" s="5"/>
-      <c r="AN19" s="5"/>
-      <c r="AO19" s="5"/>
-      <c r="AP19" s="6"/>
-      <c r="AQ19" s="6"/>
-      <c r="AR19" s="6"/>
-      <c r="AS19" s="6"/>
-      <c r="AT19" s="6"/>
-      <c r="AU19" s="6"/>
-      <c r="AV19" s="6"/>
-      <c r="AW19" s="6"/>
-      <c r="AX19" s="6"/>
-      <c r="AY19" s="6"/>
-      <c r="AZ19" s="6"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="8"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="8"/>
+      <c r="V19" s="8"/>
+      <c r="W19" s="8"/>
+      <c r="X19" s="8"/>
+      <c r="Y19" s="8"/>
+      <c r="Z19" s="8"/>
+      <c r="AA19" s="8"/>
+      <c r="AB19" s="8"/>
+      <c r="AC19" s="8"/>
+      <c r="AD19" s="8"/>
+      <c r="AE19" s="8"/>
+      <c r="AF19" s="8"/>
+      <c r="AG19" s="8"/>
+      <c r="AH19" s="8"/>
+      <c r="AI19" s="8"/>
+      <c r="AJ19" s="8"/>
+      <c r="AK19" s="8"/>
+      <c r="AL19" s="8"/>
+      <c r="AM19" s="8"/>
+      <c r="AN19" s="8"/>
+      <c r="AO19" s="8"/>
+      <c r="AP19" s="8"/>
+      <c r="AQ19" s="8"/>
+      <c r="AR19" s="8"/>
+      <c r="AS19" s="8"/>
+      <c r="AT19" s="8"/>
+      <c r="AU19" s="8"/>
+      <c r="AV19" s="8"/>
+      <c r="AW19" s="8"/>
+      <c r="AX19" s="8"/>
+      <c r="AY19" s="8"/>
+      <c r="AZ19" s="8"/>
     </row>
     <row r="20" spans="3:55" x14ac:dyDescent="0.3">
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="3"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="3"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
-      <c r="X20" s="3"/>
-      <c r="Y20" s="3"/>
-      <c r="Z20" s="3"/>
-      <c r="AA20" s="3"/>
-      <c r="AB20" s="3"/>
-      <c r="AC20" s="3"/>
-      <c r="AD20" s="3"/>
-      <c r="AE20" s="7"/>
-      <c r="AF20" s="7"/>
-      <c r="AG20" s="7"/>
-      <c r="AH20" s="7"/>
-      <c r="AI20" s="4"/>
-      <c r="AJ20" s="4"/>
-      <c r="AK20" s="4"/>
-      <c r="AL20" s="5"/>
-      <c r="AM20" s="5"/>
-      <c r="AN20" s="5"/>
-      <c r="AO20" s="5"/>
-      <c r="AP20" s="6"/>
-      <c r="AQ20" s="6"/>
-      <c r="AR20" s="6"/>
-      <c r="AS20" s="6"/>
-      <c r="AT20" s="6"/>
-      <c r="AU20" s="6"/>
-      <c r="AV20" s="6"/>
-      <c r="AW20" s="6"/>
-      <c r="AX20" s="6"/>
-      <c r="AY20" s="6"/>
-      <c r="AZ20" s="6"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+      <c r="V20" s="8"/>
+      <c r="W20" s="8"/>
+      <c r="X20" s="8"/>
+      <c r="Y20" s="8"/>
+      <c r="Z20" s="8"/>
+      <c r="AA20" s="8"/>
+      <c r="AB20" s="8"/>
+      <c r="AC20" s="8"/>
+      <c r="AD20" s="8"/>
+      <c r="AE20" s="8"/>
+      <c r="AF20" s="8"/>
+      <c r="AG20" s="8"/>
+      <c r="AH20" s="8"/>
+      <c r="AI20" s="8"/>
+      <c r="AJ20" s="8"/>
+      <c r="AK20" s="8"/>
+      <c r="AL20" s="8"/>
+      <c r="AM20" s="8"/>
+      <c r="AN20" s="8"/>
+      <c r="AO20" s="8"/>
+      <c r="AP20" s="8"/>
+      <c r="AQ20" s="8"/>
+      <c r="AR20" s="8"/>
+      <c r="AS20" s="8"/>
+      <c r="AT20" s="8"/>
+      <c r="AU20" s="8"/>
+      <c r="AV20" s="8"/>
+      <c r="AW20" s="8"/>
+      <c r="AX20" s="8"/>
+      <c r="AY20" s="8"/>
+      <c r="AZ20" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>